<commit_message>
Drop date_found and fill missing venue in prior inventory
date_found only held the Zotero import date, so it carried no
information beyond date_added. Remove it from the inventory and
from SLR-inventory.py.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/progress/SLR/prior_inventory.xlsx
+++ b/progress/SLR/prior_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git2026\research-progress\progress\SLR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56216BC2-C484-43BD-9A6A-2420ACAE49D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF533BE1-8975-41BE-82E0-78C38949E299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26460" yWindow="2985" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="119">
   <si>
     <t>id</t>
   </si>
@@ -46,9 +46,6 @@
     <t>date_added</t>
   </si>
   <si>
-    <t>date_found</t>
-  </si>
-  <si>
     <t>found_via</t>
   </si>
   <si>
@@ -79,9 +76,6 @@
     <t>2026-10-05 08:56:20</t>
   </si>
   <si>
-    <t>2026-10-05</t>
-  </si>
-  <si>
     <t>P002</t>
   </si>
   <si>
@@ -380,6 +374,9 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>Pedestrian and Evacuation Dynamics</t>
   </si>
 </sst>
 </file>
@@ -719,10 +716,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -756,414 +753,384 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
       <c r="D2">
         <v>2008</v>
       </c>
       <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
+        <v>112</v>
+      </c>
+      <c r="J2" t="s">
+        <v>115</v>
+      </c>
+      <c r="K2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>18</v>
       </c>
-      <c r="I2" t="s">
+      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="J2" t="s">
-        <v>114</v>
-      </c>
-      <c r="K2" t="s">
-        <v>117</v>
-      </c>
-      <c r="L2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="C3" t="s">
         <v>20</v>
-      </c>
-      <c r="B3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
       </c>
       <c r="D3">
         <v>2008</v>
       </c>
       <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" t="s">
+        <v>118</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
         <v>23</v>
       </c>
-      <c r="G3" t="s">
-        <v>24</v>
-      </c>
-      <c r="H3" t="s">
-        <v>25</v>
-      </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="J3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K3" t="s">
         <v>117</v>
       </c>
-      <c r="L3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
         <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" t="s">
-        <v>28</v>
       </c>
       <c r="D4">
         <v>2013</v>
       </c>
       <c r="E4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>30</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J4" t="s">
+        <v>115</v>
+      </c>
+      <c r="K4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>31</v>
       </c>
-      <c r="H4" t="s">
+      <c r="B5" t="s">
         <v>32</v>
       </c>
-      <c r="I4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" t="s">
-        <v>114</v>
-      </c>
-      <c r="K4" t="s">
-        <v>117</v>
-      </c>
-      <c r="L4" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C5" t="s">
         <v>33</v>
-      </c>
-      <c r="B5" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" t="s">
-        <v>35</v>
       </c>
       <c r="D5">
         <v>2014</v>
       </c>
       <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" t="s">
         <v>36</v>
       </c>
-      <c r="F5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" t="s">
-        <v>37</v>
-      </c>
-      <c r="H5" t="s">
-        <v>38</v>
-      </c>
       <c r="I5" t="s">
-        <v>19</v>
+        <v>113</v>
       </c>
       <c r="J5" t="s">
         <v>115</v>
       </c>
       <c r="K5" t="s">
-        <v>117</v>
-      </c>
-      <c r="L5" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
         <v>39</v>
-      </c>
-      <c r="B6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" t="s">
-        <v>41</v>
       </c>
       <c r="D6">
         <v>2015</v>
       </c>
       <c r="E6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
         <v>42</v>
       </c>
-      <c r="F6" t="s">
+      <c r="H6" t="s">
         <v>43</v>
       </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
+        <v>112</v>
+      </c>
+      <c r="J6" t="s">
+        <v>115</v>
+      </c>
+      <c r="K6" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>44</v>
       </c>
-      <c r="H6" t="s">
+      <c r="B7" t="s">
         <v>45</v>
       </c>
-      <c r="I6" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" t="s">
-        <v>114</v>
-      </c>
-      <c r="K6" t="s">
-        <v>117</v>
-      </c>
-      <c r="L6" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C7" t="s">
         <v>46</v>
-      </c>
-      <c r="B7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" t="s">
-        <v>48</v>
       </c>
       <c r="D7">
         <v>2016</v>
       </c>
       <c r="E7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" t="s">
         <v>49</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>50</v>
       </c>
-      <c r="G7" t="s">
-        <v>51</v>
-      </c>
-      <c r="H7" t="s">
-        <v>52</v>
-      </c>
       <c r="I7" t="s">
-        <v>19</v>
+        <v>113</v>
       </c>
       <c r="J7" t="s">
         <v>115</v>
       </c>
       <c r="K7" t="s">
-        <v>117</v>
-      </c>
-      <c r="L7" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
         <v>53</v>
-      </c>
-      <c r="B8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C8" t="s">
-        <v>55</v>
       </c>
       <c r="D8">
         <v>2017</v>
       </c>
       <c r="E8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" t="s">
         <v>56</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>57</v>
       </c>
-      <c r="G8" t="s">
+      <c r="I8" t="s">
+        <v>112</v>
+      </c>
+      <c r="J8" t="s">
+        <v>115</v>
+      </c>
+      <c r="K8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>58</v>
       </c>
-      <c r="H8" t="s">
+      <c r="B9" t="s">
         <v>59</v>
       </c>
-      <c r="I8" t="s">
-        <v>19</v>
-      </c>
-      <c r="J8" t="s">
-        <v>114</v>
-      </c>
-      <c r="K8" t="s">
-        <v>117</v>
-      </c>
-      <c r="L8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
         <v>60</v>
-      </c>
-      <c r="B9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" t="s">
-        <v>62</v>
       </c>
       <c r="D9">
         <v>2019</v>
       </c>
       <c r="E9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" t="s">
         <v>63</v>
       </c>
-      <c r="F9" t="s">
+      <c r="H9" t="s">
         <v>64</v>
       </c>
-      <c r="G9" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" t="s">
-        <v>66</v>
-      </c>
       <c r="I9" t="s">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="J9" t="s">
         <v>114</v>
       </c>
       <c r="K9" t="s">
-        <v>116</v>
-      </c>
-      <c r="L9" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" t="s">
         <v>67</v>
-      </c>
-      <c r="B10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C10" t="s">
-        <v>69</v>
       </c>
       <c r="D10">
         <v>2023</v>
       </c>
       <c r="E10" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" t="s">
+        <v>69</v>
+      </c>
+      <c r="H10" t="s">
         <v>70</v>
       </c>
-      <c r="F10" t="s">
-        <v>64</v>
-      </c>
-      <c r="G10" t="s">
-        <v>71</v>
-      </c>
-      <c r="H10" t="s">
-        <v>72</v>
-      </c>
       <c r="I10" t="s">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="J10" t="s">
         <v>114</v>
       </c>
       <c r="K10" t="s">
-        <v>116</v>
-      </c>
-      <c r="L10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" t="s">
         <v>73</v>
-      </c>
-      <c r="B11" t="s">
-        <v>74</v>
-      </c>
-      <c r="C11" t="s">
-        <v>75</v>
       </c>
       <c r="D11">
         <v>2023</v>
       </c>
       <c r="E11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" t="s">
         <v>76</v>
       </c>
-      <c r="F11" t="s">
+      <c r="H11" t="s">
         <v>77</v>
       </c>
-      <c r="G11" t="s">
-        <v>78</v>
-      </c>
-      <c r="H11" t="s">
-        <v>79</v>
-      </c>
       <c r="I11" t="s">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="J11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K11" t="s">
         <v>117</v>
       </c>
-      <c r="L11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" t="s">
         <v>80</v>
-      </c>
-      <c r="B12" t="s">
-        <v>81</v>
-      </c>
-      <c r="C12" t="s">
-        <v>82</v>
       </c>
       <c r="D12">
         <v>2023</v>
       </c>
       <c r="E12" t="s">
+        <v>81</v>
+      </c>
+      <c r="F12" t="s">
+        <v>82</v>
+      </c>
+      <c r="G12" t="s">
         <v>83</v>
       </c>
-      <c r="F12" t="s">
+      <c r="H12" t="s">
         <v>84</v>
       </c>
-      <c r="G12" t="s">
-        <v>85</v>
-      </c>
-      <c r="H12" t="s">
-        <v>86</v>
-      </c>
       <c r="I12" t="s">
-        <v>19</v>
+        <v>113</v>
       </c>
       <c r="J12" t="s">
         <v>115</v>
@@ -1171,160 +1138,145 @@
       <c r="K12" t="s">
         <v>117</v>
       </c>
-      <c r="L12" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" t="s">
         <v>87</v>
-      </c>
-      <c r="B13" t="s">
-        <v>88</v>
-      </c>
-      <c r="C13" t="s">
-        <v>89</v>
       </c>
       <c r="D13">
         <v>2025</v>
       </c>
       <c r="E13" t="s">
+        <v>88</v>
+      </c>
+      <c r="F13" t="s">
+        <v>62</v>
+      </c>
+      <c r="G13" t="s">
+        <v>89</v>
+      </c>
+      <c r="H13" t="s">
         <v>90</v>
       </c>
-      <c r="F13" t="s">
-        <v>64</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="I13" t="s">
+        <v>112</v>
+      </c>
+      <c r="J13" t="s">
+        <v>115</v>
+      </c>
+      <c r="K13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>91</v>
       </c>
-      <c r="H13" t="s">
+      <c r="B14" t="s">
         <v>92</v>
       </c>
-      <c r="I13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J13" t="s">
-        <v>114</v>
-      </c>
-      <c r="K13" t="s">
-        <v>117</v>
-      </c>
-      <c r="L13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="C14" t="s">
         <v>93</v>
-      </c>
-      <c r="B14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C14" t="s">
-        <v>95</v>
       </c>
       <c r="D14">
         <v>2025</v>
       </c>
       <c r="E14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F14" t="s">
+        <v>95</v>
+      </c>
+      <c r="G14" t="s">
         <v>96</v>
       </c>
-      <c r="F14" t="s">
+      <c r="H14" t="s">
         <v>97</v>
       </c>
-      <c r="G14" t="s">
-        <v>98</v>
-      </c>
-      <c r="H14" t="s">
-        <v>99</v>
-      </c>
       <c r="I14" t="s">
-        <v>19</v>
+        <v>112</v>
       </c>
       <c r="J14" t="s">
         <v>114</v>
       </c>
       <c r="K14" t="s">
-        <v>116</v>
-      </c>
-      <c r="L14" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15" t="s">
         <v>100</v>
-      </c>
-      <c r="B15" t="s">
-        <v>101</v>
-      </c>
-      <c r="C15" t="s">
-        <v>102</v>
       </c>
       <c r="D15">
         <v>2025</v>
       </c>
       <c r="E15" t="s">
+        <v>101</v>
+      </c>
+      <c r="F15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G15" t="s">
         <v>103</v>
       </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>104</v>
       </c>
-      <c r="G15" t="s">
+      <c r="I15" t="s">
+        <v>112</v>
+      </c>
+      <c r="J15" t="s">
+        <v>115</v>
+      </c>
+      <c r="K15" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>105</v>
       </c>
-      <c r="H15" t="s">
+      <c r="B16" t="s">
         <v>106</v>
       </c>
-      <c r="I15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J15" t="s">
-        <v>114</v>
-      </c>
-      <c r="K15" t="s">
-        <v>117</v>
-      </c>
-      <c r="L15" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="C16" t="s">
         <v>107</v>
-      </c>
-      <c r="B16" t="s">
-        <v>108</v>
-      </c>
-      <c r="C16" t="s">
-        <v>109</v>
       </c>
       <c r="D16">
         <v>2026</v>
       </c>
       <c r="E16" t="s">
+        <v>108</v>
+      </c>
+      <c r="F16" t="s">
+        <v>109</v>
+      </c>
+      <c r="G16" t="s">
         <v>110</v>
       </c>
-      <c r="F16" t="s">
+      <c r="H16" t="s">
         <v>111</v>
       </c>
-      <c r="G16" t="s">
+      <c r="I16" t="s">
         <v>112</v>
       </c>
-      <c r="H16" t="s">
-        <v>113</v>
-      </c>
-      <c r="I16" t="s">
-        <v>19</v>
-      </c>
       <c r="J16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K16" t="s">
         <v>117</v>
-      </c>
-      <c r="L16" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>